<commit_message>
data files for game events added dictionary updated
</commit_message>
<xml_diff>
--- a/2025-2026/Data/Data_Dictionary.xlsx
+++ b/2025-2026/Data/Data_Dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alex\Documents\NHL-Stats\2025-2026\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF726EEA-0D18-4160-8039-8AE1491954D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE3554E4-538B-4B9E-A20C-3D2040C64C11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43095" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{63DB0C7C-412E-4A18-A7BF-880A50C6E4C7}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{63DB0C7C-412E-4A18-A7BF-880A50C6E4C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="160">
   <si>
     <t>Variable</t>
   </si>
@@ -351,6 +351,174 @@
   </si>
   <si>
     <t xml:space="preserve">id of the player who won the faceoff </t>
+  </si>
+  <si>
+    <t>shot_type</t>
+  </si>
+  <si>
+    <t>shoot_player_id</t>
+  </si>
+  <si>
+    <t>goalie_in_id</t>
+  </si>
+  <si>
+    <t>away_sog</t>
+  </si>
+  <si>
+    <t>home_sog</t>
+  </si>
+  <si>
+    <t>miss_reason</t>
+  </si>
+  <si>
+    <t>block_player_id</t>
+  </si>
+  <si>
+    <t>block_reason</t>
+  </si>
+  <si>
+    <t>all_shots</t>
+  </si>
+  <si>
+    <t>blocked_shots</t>
+  </si>
+  <si>
+    <t>id of the player who shot the puck</t>
+  </si>
+  <si>
+    <t>id of the player who blocked the shot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">type of block: blocked, teammate blocked, other block </t>
+  </si>
+  <si>
+    <t>missed_shots</t>
+  </si>
+  <si>
+    <t>Type of shot: backhand, bat, between-legs, cradle, deflected, poke, slap, snap, tip-in, wrap-around, wrist</t>
+  </si>
+  <si>
+    <t>reason for the miss attempt: above-crossbar, failed-bank-attempt, high-and-wide-left, high-and-wide-right, hit-crossbar, hit-left-post, hit-right-post, short, wide-left, wide-right</t>
+  </si>
+  <si>
+    <t>shots_on_goal</t>
+  </si>
+  <si>
+    <t>id of the goalie who was in net and made the save on the shot</t>
+  </si>
+  <si>
+    <t>total number of shots on goal for the away team when the current shot was taken</t>
+  </si>
+  <si>
+    <t>total number of shots on goal for the home team when the current shot was taken</t>
+  </si>
+  <si>
+    <t>give_player_id</t>
+  </si>
+  <si>
+    <t>giveaways</t>
+  </si>
+  <si>
+    <t>id of the player who is charged with the giveaway</t>
+  </si>
+  <si>
+    <t>score_player_id</t>
+  </si>
+  <si>
+    <t>score_player_total</t>
+  </si>
+  <si>
+    <t>assist_1_player_id</t>
+  </si>
+  <si>
+    <t>assist_1_player_total</t>
+  </si>
+  <si>
+    <t>assist_2_player_id</t>
+  </si>
+  <si>
+    <t>assist_2_player_total</t>
+  </si>
+  <si>
+    <t>away_score</t>
+  </si>
+  <si>
+    <t>home_score</t>
+  </si>
+  <si>
+    <t>video_link</t>
+  </si>
+  <si>
+    <t>goals</t>
+  </si>
+  <si>
+    <t>id of the goalie who was in net for the goal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id of the player who scored the goal </t>
+  </si>
+  <si>
+    <t>total number of goals for the goal scorer on the season</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id of the player who has the primary assist on the goal </t>
+  </si>
+  <si>
+    <t xml:space="preserve">total number of assists on the season for the player with the primary assist </t>
+  </si>
+  <si>
+    <t xml:space="preserve">id of the player who has the secondary assist on the goal </t>
+  </si>
+  <si>
+    <t xml:space="preserve">total number of assists on the season for the player with the secondary assist </t>
+  </si>
+  <si>
+    <t>score for the away team at the time of the goal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">score for the home team at the time of the goal </t>
+  </si>
+  <si>
+    <t xml:space="preserve">link t o video of the goal </t>
+  </si>
+  <si>
+    <t>hitter_id</t>
+  </si>
+  <si>
+    <t>hittee_id</t>
+  </si>
+  <si>
+    <t>hits</t>
+  </si>
+  <si>
+    <t>id of the player who made the hit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id of the player who was hit </t>
+  </si>
+  <si>
+    <t>take_player_id</t>
+  </si>
+  <si>
+    <t>takeaways</t>
+  </si>
+  <si>
+    <t>id of the player who was awarded with the takeaway</t>
+  </si>
+  <si>
+    <t>team_id</t>
+  </si>
+  <si>
+    <t>team</t>
+  </si>
+  <si>
+    <t>teams</t>
+  </si>
+  <si>
+    <t>numerical code indicating the team</t>
+  </si>
+  <si>
+    <t>3-letter code indicating the team name</t>
   </si>
 </sst>
 </file>
@@ -731,10 +899,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94ACE342-EFD3-426B-82E7-62E8481985EA}">
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C204"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.44140625" customWidth="1"/>
     <col min="3" max="3" width="85.21875" customWidth="1"/>
   </cols>
@@ -1443,6 +1611,1546 @@
         <v>103</v>
       </c>
     </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>2</v>
+      </c>
+      <c r="B65" t="s">
+        <v>112</v>
+      </c>
+      <c r="C65" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>64</v>
+      </c>
+      <c r="B66" t="s">
+        <v>112</v>
+      </c>
+      <c r="C66" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>65</v>
+      </c>
+      <c r="B67" t="s">
+        <v>112</v>
+      </c>
+      <c r="C67" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>66</v>
+      </c>
+      <c r="B68" t="s">
+        <v>112</v>
+      </c>
+      <c r="C68" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>67</v>
+      </c>
+      <c r="B69" t="s">
+        <v>112</v>
+      </c>
+      <c r="C69" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>68</v>
+      </c>
+      <c r="B70" t="s">
+        <v>112</v>
+      </c>
+      <c r="C70" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>69</v>
+      </c>
+      <c r="B71" t="s">
+        <v>112</v>
+      </c>
+      <c r="C71" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>70</v>
+      </c>
+      <c r="B72" t="s">
+        <v>112</v>
+      </c>
+      <c r="C72" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>71</v>
+      </c>
+      <c r="B73" t="s">
+        <v>112</v>
+      </c>
+      <c r="C73" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>72</v>
+      </c>
+      <c r="B74" t="s">
+        <v>112</v>
+      </c>
+      <c r="C74" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>73</v>
+      </c>
+      <c r="B75" t="s">
+        <v>112</v>
+      </c>
+      <c r="C75" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>74</v>
+      </c>
+      <c r="B76" t="s">
+        <v>112</v>
+      </c>
+      <c r="C76" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>75</v>
+      </c>
+      <c r="B77" t="s">
+        <v>112</v>
+      </c>
+      <c r="C77" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>104</v>
+      </c>
+      <c r="B78" t="s">
+        <v>112</v>
+      </c>
+      <c r="C78" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>105</v>
+      </c>
+      <c r="B79" t="s">
+        <v>112</v>
+      </c>
+      <c r="C79" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>106</v>
+      </c>
+      <c r="B80" t="s">
+        <v>112</v>
+      </c>
+      <c r="C80" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>107</v>
+      </c>
+      <c r="B81" t="s">
+        <v>112</v>
+      </c>
+      <c r="C81" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>108</v>
+      </c>
+      <c r="B82" t="s">
+        <v>112</v>
+      </c>
+      <c r="C82" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>109</v>
+      </c>
+      <c r="B83" t="s">
+        <v>112</v>
+      </c>
+      <c r="C83" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>110</v>
+      </c>
+      <c r="B84" t="s">
+        <v>112</v>
+      </c>
+      <c r="C84" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>111</v>
+      </c>
+      <c r="B85" t="s">
+        <v>112</v>
+      </c>
+      <c r="C85" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>2</v>
+      </c>
+      <c r="B86" t="s">
+        <v>113</v>
+      </c>
+      <c r="C86" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>64</v>
+      </c>
+      <c r="B87" t="s">
+        <v>113</v>
+      </c>
+      <c r="C87" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>65</v>
+      </c>
+      <c r="B88" t="s">
+        <v>113</v>
+      </c>
+      <c r="C88" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>66</v>
+      </c>
+      <c r="B89" t="s">
+        <v>113</v>
+      </c>
+      <c r="C89" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>67</v>
+      </c>
+      <c r="B90" t="s">
+        <v>113</v>
+      </c>
+      <c r="C90" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>68</v>
+      </c>
+      <c r="B91" t="s">
+        <v>113</v>
+      </c>
+      <c r="C91" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>69</v>
+      </c>
+      <c r="B92" t="s">
+        <v>113</v>
+      </c>
+      <c r="C92" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>70</v>
+      </c>
+      <c r="B93" t="s">
+        <v>113</v>
+      </c>
+      <c r="C93" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>71</v>
+      </c>
+      <c r="B94" t="s">
+        <v>113</v>
+      </c>
+      <c r="C94" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>72</v>
+      </c>
+      <c r="B95" t="s">
+        <v>113</v>
+      </c>
+      <c r="C95" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>73</v>
+      </c>
+      <c r="B96" t="s">
+        <v>113</v>
+      </c>
+      <c r="C96" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>74</v>
+      </c>
+      <c r="B97" t="s">
+        <v>113</v>
+      </c>
+      <c r="C97" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>75</v>
+      </c>
+      <c r="B98" t="s">
+        <v>113</v>
+      </c>
+      <c r="C98" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>105</v>
+      </c>
+      <c r="B99" t="s">
+        <v>113</v>
+      </c>
+      <c r="C99" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>110</v>
+      </c>
+      <c r="B100" t="s">
+        <v>113</v>
+      </c>
+      <c r="C100" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>111</v>
+      </c>
+      <c r="B101" t="s">
+        <v>113</v>
+      </c>
+      <c r="C101" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>2</v>
+      </c>
+      <c r="B102" t="s">
+        <v>117</v>
+      </c>
+      <c r="C102" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>64</v>
+      </c>
+      <c r="B103" t="s">
+        <v>117</v>
+      </c>
+      <c r="C103" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>65</v>
+      </c>
+      <c r="B104" t="s">
+        <v>117</v>
+      </c>
+      <c r="C104" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A105" t="s">
+        <v>66</v>
+      </c>
+      <c r="B105" t="s">
+        <v>117</v>
+      </c>
+      <c r="C105" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A106" t="s">
+        <v>67</v>
+      </c>
+      <c r="B106" t="s">
+        <v>117</v>
+      </c>
+      <c r="C106" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A107" t="s">
+        <v>68</v>
+      </c>
+      <c r="B107" t="s">
+        <v>117</v>
+      </c>
+      <c r="C107" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
+        <v>69</v>
+      </c>
+      <c r="B108" t="s">
+        <v>117</v>
+      </c>
+      <c r="C108" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A109" t="s">
+        <v>70</v>
+      </c>
+      <c r="B109" t="s">
+        <v>117</v>
+      </c>
+      <c r="C109" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A110" t="s">
+        <v>71</v>
+      </c>
+      <c r="B110" t="s">
+        <v>117</v>
+      </c>
+      <c r="C110" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A111" t="s">
+        <v>72</v>
+      </c>
+      <c r="B111" t="s">
+        <v>117</v>
+      </c>
+      <c r="C111" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A112" t="s">
+        <v>73</v>
+      </c>
+      <c r="B112" t="s">
+        <v>117</v>
+      </c>
+      <c r="C112" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
+        <v>74</v>
+      </c>
+      <c r="B113" t="s">
+        <v>117</v>
+      </c>
+      <c r="C113" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A114" t="s">
+        <v>75</v>
+      </c>
+      <c r="B114" t="s">
+        <v>117</v>
+      </c>
+      <c r="C114" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A115" t="s">
+        <v>104</v>
+      </c>
+      <c r="B115" t="s">
+        <v>117</v>
+      </c>
+      <c r="C115" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A116" t="s">
+        <v>105</v>
+      </c>
+      <c r="B116" t="s">
+        <v>117</v>
+      </c>
+      <c r="C116" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A117" t="s">
+        <v>109</v>
+      </c>
+      <c r="B117" t="s">
+        <v>117</v>
+      </c>
+      <c r="C117" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A118" t="s">
+        <v>2</v>
+      </c>
+      <c r="B118" t="s">
+        <v>120</v>
+      </c>
+      <c r="C118" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A119" t="s">
+        <v>64</v>
+      </c>
+      <c r="B119" t="s">
+        <v>120</v>
+      </c>
+      <c r="C119" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A120" t="s">
+        <v>65</v>
+      </c>
+      <c r="B120" t="s">
+        <v>120</v>
+      </c>
+      <c r="C120" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A121" t="s">
+        <v>66</v>
+      </c>
+      <c r="B121" t="s">
+        <v>120</v>
+      </c>
+      <c r="C121" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A122" t="s">
+        <v>67</v>
+      </c>
+      <c r="B122" t="s">
+        <v>120</v>
+      </c>
+      <c r="C122" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A123" t="s">
+        <v>68</v>
+      </c>
+      <c r="B123" t="s">
+        <v>120</v>
+      </c>
+      <c r="C123" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A124" t="s">
+        <v>69</v>
+      </c>
+      <c r="B124" t="s">
+        <v>120</v>
+      </c>
+      <c r="C124" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A125" t="s">
+        <v>70</v>
+      </c>
+      <c r="B125" t="s">
+        <v>120</v>
+      </c>
+      <c r="C125" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A126" t="s">
+        <v>71</v>
+      </c>
+      <c r="B126" t="s">
+        <v>120</v>
+      </c>
+      <c r="C126" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A127" t="s">
+        <v>72</v>
+      </c>
+      <c r="B127" t="s">
+        <v>120</v>
+      </c>
+      <c r="C127" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A128" t="s">
+        <v>73</v>
+      </c>
+      <c r="B128" t="s">
+        <v>120</v>
+      </c>
+      <c r="C128" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A129" t="s">
+        <v>74</v>
+      </c>
+      <c r="B129" t="s">
+        <v>120</v>
+      </c>
+      <c r="C129" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A130" t="s">
+        <v>75</v>
+      </c>
+      <c r="B130" t="s">
+        <v>120</v>
+      </c>
+      <c r="C130" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A131" t="s">
+        <v>104</v>
+      </c>
+      <c r="B131" t="s">
+        <v>120</v>
+      </c>
+      <c r="C131" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A132" t="s">
+        <v>105</v>
+      </c>
+      <c r="B132" t="s">
+        <v>120</v>
+      </c>
+      <c r="C132" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A133" t="s">
+        <v>106</v>
+      </c>
+      <c r="B133" t="s">
+        <v>120</v>
+      </c>
+      <c r="C133" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A134" t="s">
+        <v>107</v>
+      </c>
+      <c r="B134" t="s">
+        <v>120</v>
+      </c>
+      <c r="C134" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A135" t="s">
+        <v>108</v>
+      </c>
+      <c r="B135" t="s">
+        <v>120</v>
+      </c>
+      <c r="C135" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A136" t="s">
+        <v>2</v>
+      </c>
+      <c r="B136" t="s">
+        <v>125</v>
+      </c>
+      <c r="C136" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A137" t="s">
+        <v>64</v>
+      </c>
+      <c r="B137" t="s">
+        <v>125</v>
+      </c>
+      <c r="C137" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A138" t="s">
+        <v>65</v>
+      </c>
+      <c r="B138" t="s">
+        <v>125</v>
+      </c>
+      <c r="C138" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A139" t="s">
+        <v>66</v>
+      </c>
+      <c r="B139" t="s">
+        <v>125</v>
+      </c>
+      <c r="C139" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A140" t="s">
+        <v>67</v>
+      </c>
+      <c r="B140" t="s">
+        <v>125</v>
+      </c>
+      <c r="C140" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A141" t="s">
+        <v>68</v>
+      </c>
+      <c r="B141" t="s">
+        <v>125</v>
+      </c>
+      <c r="C141" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A142" t="s">
+        <v>69</v>
+      </c>
+      <c r="B142" t="s">
+        <v>125</v>
+      </c>
+      <c r="C142" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A143" t="s">
+        <v>70</v>
+      </c>
+      <c r="B143" t="s">
+        <v>125</v>
+      </c>
+      <c r="C143" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A144" t="s">
+        <v>71</v>
+      </c>
+      <c r="B144" t="s">
+        <v>125</v>
+      </c>
+      <c r="C144" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A145" t="s">
+        <v>72</v>
+      </c>
+      <c r="B145" t="s">
+        <v>125</v>
+      </c>
+      <c r="C145" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A146" t="s">
+        <v>73</v>
+      </c>
+      <c r="B146" t="s">
+        <v>125</v>
+      </c>
+      <c r="C146" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A147" t="s">
+        <v>74</v>
+      </c>
+      <c r="B147" t="s">
+        <v>125</v>
+      </c>
+      <c r="C147" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A148" t="s">
+        <v>75</v>
+      </c>
+      <c r="B148" t="s">
+        <v>125</v>
+      </c>
+      <c r="C148" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A149" t="s">
+        <v>124</v>
+      </c>
+      <c r="B149" t="s">
+        <v>125</v>
+      </c>
+      <c r="C149" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A150" t="s">
+        <v>2</v>
+      </c>
+      <c r="B150" t="s">
+        <v>136</v>
+      </c>
+      <c r="C150" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A151" t="s">
+        <v>64</v>
+      </c>
+      <c r="B151" t="s">
+        <v>136</v>
+      </c>
+      <c r="C151" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A152" t="s">
+        <v>65</v>
+      </c>
+      <c r="B152" t="s">
+        <v>136</v>
+      </c>
+      <c r="C152" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A153" t="s">
+        <v>66</v>
+      </c>
+      <c r="B153" t="s">
+        <v>136</v>
+      </c>
+      <c r="C153" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A154" t="s">
+        <v>67</v>
+      </c>
+      <c r="B154" t="s">
+        <v>136</v>
+      </c>
+      <c r="C154" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A155" t="s">
+        <v>68</v>
+      </c>
+      <c r="B155" t="s">
+        <v>136</v>
+      </c>
+      <c r="C155" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A156" t="s">
+        <v>69</v>
+      </c>
+      <c r="B156" t="s">
+        <v>136</v>
+      </c>
+      <c r="C156" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A157" t="s">
+        <v>70</v>
+      </c>
+      <c r="B157" t="s">
+        <v>136</v>
+      </c>
+      <c r="C157" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A158" t="s">
+        <v>71</v>
+      </c>
+      <c r="B158" t="s">
+        <v>136</v>
+      </c>
+      <c r="C158" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A159" t="s">
+        <v>72</v>
+      </c>
+      <c r="B159" t="s">
+        <v>136</v>
+      </c>
+      <c r="C159" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A160" t="s">
+        <v>73</v>
+      </c>
+      <c r="B160" t="s">
+        <v>136</v>
+      </c>
+      <c r="C160" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A161" t="s">
+        <v>74</v>
+      </c>
+      <c r="B161" t="s">
+        <v>136</v>
+      </c>
+      <c r="C161" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A162" t="s">
+        <v>75</v>
+      </c>
+      <c r="B162" t="s">
+        <v>136</v>
+      </c>
+      <c r="C162" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A163" t="s">
+        <v>104</v>
+      </c>
+      <c r="B163" t="s">
+        <v>136</v>
+      </c>
+      <c r="C163" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A164" t="s">
+        <v>106</v>
+      </c>
+      <c r="B164" t="s">
+        <v>136</v>
+      </c>
+      <c r="C164" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A165" t="s">
+        <v>127</v>
+      </c>
+      <c r="B165" t="s">
+        <v>136</v>
+      </c>
+      <c r="C165" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A166" t="s">
+        <v>128</v>
+      </c>
+      <c r="B166" t="s">
+        <v>136</v>
+      </c>
+      <c r="C166" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A167" t="s">
+        <v>129</v>
+      </c>
+      <c r="B167" t="s">
+        <v>136</v>
+      </c>
+      <c r="C167" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A168" t="s">
+        <v>130</v>
+      </c>
+      <c r="B168" t="s">
+        <v>136</v>
+      </c>
+      <c r="C168" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="169" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A169" t="s">
+        <v>131</v>
+      </c>
+      <c r="B169" t="s">
+        <v>136</v>
+      </c>
+      <c r="C169" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="170" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A170" t="s">
+        <v>132</v>
+      </c>
+      <c r="B170" t="s">
+        <v>136</v>
+      </c>
+      <c r="C170" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A171" t="s">
+        <v>133</v>
+      </c>
+      <c r="B171" t="s">
+        <v>136</v>
+      </c>
+      <c r="C171" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A172" t="s">
+        <v>134</v>
+      </c>
+      <c r="B172" t="s">
+        <v>136</v>
+      </c>
+      <c r="C172" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A173" t="s">
+        <v>135</v>
+      </c>
+      <c r="B173" t="s">
+        <v>136</v>
+      </c>
+      <c r="C173" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A174" t="s">
+        <v>2</v>
+      </c>
+      <c r="B174" t="s">
+        <v>149</v>
+      </c>
+      <c r="C174" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A175" t="s">
+        <v>64</v>
+      </c>
+      <c r="B175" t="s">
+        <v>149</v>
+      </c>
+      <c r="C175" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A176" t="s">
+        <v>65</v>
+      </c>
+      <c r="B176" t="s">
+        <v>149</v>
+      </c>
+      <c r="C176" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A177" t="s">
+        <v>66</v>
+      </c>
+      <c r="B177" t="s">
+        <v>149</v>
+      </c>
+      <c r="C177" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A178" t="s">
+        <v>67</v>
+      </c>
+      <c r="B178" t="s">
+        <v>149</v>
+      </c>
+      <c r="C178" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A179" t="s">
+        <v>68</v>
+      </c>
+      <c r="B179" t="s">
+        <v>149</v>
+      </c>
+      <c r="C179" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A180" t="s">
+        <v>69</v>
+      </c>
+      <c r="B180" t="s">
+        <v>149</v>
+      </c>
+      <c r="C180" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A181" t="s">
+        <v>70</v>
+      </c>
+      <c r="B181" t="s">
+        <v>149</v>
+      </c>
+      <c r="C181" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A182" t="s">
+        <v>71</v>
+      </c>
+      <c r="B182" t="s">
+        <v>149</v>
+      </c>
+      <c r="C182" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A183" t="s">
+        <v>72</v>
+      </c>
+      <c r="B183" t="s">
+        <v>149</v>
+      </c>
+      <c r="C183" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A184" t="s">
+        <v>73</v>
+      </c>
+      <c r="B184" t="s">
+        <v>149</v>
+      </c>
+      <c r="C184" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A185" t="s">
+        <v>74</v>
+      </c>
+      <c r="B185" t="s">
+        <v>149</v>
+      </c>
+      <c r="C185" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A186" t="s">
+        <v>75</v>
+      </c>
+      <c r="B186" t="s">
+        <v>149</v>
+      </c>
+      <c r="C186" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A187" t="s">
+        <v>147</v>
+      </c>
+      <c r="B187" t="s">
+        <v>149</v>
+      </c>
+      <c r="C187" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A188" t="s">
+        <v>148</v>
+      </c>
+      <c r="B188" t="s">
+        <v>149</v>
+      </c>
+      <c r="C188" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A189" t="s">
+        <v>2</v>
+      </c>
+      <c r="B189" t="s">
+        <v>153</v>
+      </c>
+      <c r="C189" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="190" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A190" t="s">
+        <v>64</v>
+      </c>
+      <c r="B190" t="s">
+        <v>153</v>
+      </c>
+      <c r="C190" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A191" t="s">
+        <v>65</v>
+      </c>
+      <c r="B191" t="s">
+        <v>153</v>
+      </c>
+      <c r="C191" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A192" t="s">
+        <v>66</v>
+      </c>
+      <c r="B192" t="s">
+        <v>153</v>
+      </c>
+      <c r="C192" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A193" t="s">
+        <v>67</v>
+      </c>
+      <c r="B193" t="s">
+        <v>153</v>
+      </c>
+      <c r="C193" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A194" t="s">
+        <v>68</v>
+      </c>
+      <c r="B194" t="s">
+        <v>153</v>
+      </c>
+      <c r="C194" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="195" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A195" t="s">
+        <v>69</v>
+      </c>
+      <c r="B195" t="s">
+        <v>153</v>
+      </c>
+      <c r="C195" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A196" t="s">
+        <v>70</v>
+      </c>
+      <c r="B196" t="s">
+        <v>153</v>
+      </c>
+      <c r="C196" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A197" t="s">
+        <v>71</v>
+      </c>
+      <c r="B197" t="s">
+        <v>153</v>
+      </c>
+      <c r="C197" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A198" t="s">
+        <v>72</v>
+      </c>
+      <c r="B198" t="s">
+        <v>153</v>
+      </c>
+      <c r="C198" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="199" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A199" t="s">
+        <v>73</v>
+      </c>
+      <c r="B199" t="s">
+        <v>153</v>
+      </c>
+      <c r="C199" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="200" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A200" t="s">
+        <v>74</v>
+      </c>
+      <c r="B200" t="s">
+        <v>153</v>
+      </c>
+      <c r="C200" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A201" t="s">
+        <v>75</v>
+      </c>
+      <c r="B201" t="s">
+        <v>153</v>
+      </c>
+      <c r="C201" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="202" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A202" t="s">
+        <v>152</v>
+      </c>
+      <c r="B202" t="s">
+        <v>153</v>
+      </c>
+      <c r="C202" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="203" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A203" t="s">
+        <v>155</v>
+      </c>
+      <c r="B203" t="s">
+        <v>157</v>
+      </c>
+      <c r="C203" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="204" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A204" t="s">
+        <v>156</v>
+      </c>
+      <c r="B204" t="s">
+        <v>157</v>
+      </c>
+      <c r="C204" t="s">
+        <v>159</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>